<commit_message>
chore: update release/v2026.4.0 pages
</commit_message>
<xml_diff>
--- a/release/v2026.4.0/CodeSystem-mii-cs-pro-bdi-bdi2.xlsx
+++ b/release/v2026.4.0/CodeSystem-mii-cs-pro-bdi-bdi2.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2026.2.0</t>
+    <t>2026.4.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-14T19:09:51+00:00</t>
+    <t>2026-06-14T19:15:38+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>